<commit_message>
Musique : mention d'auteur et coups de cœur YouTube Music
- Colonne « auteur » facultative dans musique.xlsx, affichée « Morceau de … » (Schwarze Rose de Cadidscha)
- Section « Mes coups de cœur » avec lecteur YouTube intégré (data/coups-de-coeur.json)

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/data/musique.xlsx
+++ b/data/musique.xlsx
@@ -21,7 +21,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="22" uniqueCount="22">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="25" uniqueCount="25">
   <si>
     <t>titre</t>
   </si>
@@ -87,6 +87,15 @@
   </si>
   <si>
     <t>Darkwave</t>
+  </si>
+  <si>
+    <t>auteur</t>
+  </si>
+  <si>
+    <t>Cadidscha</t>
+  </si>
+  <si>
+    <t>auteur : facultatif. Laisse vide pour tes propres morceaux ; sinon indique le nom de l’auteur (ex. Cadidscha), affiché sur le site.</t>
   </si>
 </sst>
 </file>
@@ -160,14 +169,15 @@
 </file>
 
 <file path=xl/tables/table1.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="1" xr:uid="{00000000-000C-0000-FFFF-FFFF00000000}" name="Morceaux" displayName="Morceaux" ref="A1:E13">
-  <autoFilter ref="A1:E13" xr:uid="{00000000-0009-0000-0100-000001000000}"/>
-  <tableColumns count="5">
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="1" xr:uid="{00000000-000C-0000-FFFF-FFFF00000000}" name="Morceaux" displayName="Morceaux" ref="A1:F13">
+  <autoFilter ref="A1:F13" xr:uid="{00000000-0009-0000-0100-000001000000}"/>
+  <tableColumns count="6">
     <tableColumn id="1" xr3:uid="{00000000-0010-0000-0000-000001000000}" name="titre"/>
     <tableColumn id="2" xr3:uid="{00000000-0010-0000-0000-000002000000}" name="style"/>
     <tableColumn id="3" xr3:uid="{00000000-0010-0000-0000-000003000000}" name="date"/>
     <tableColumn id="4" xr3:uid="{00000000-0010-0000-0000-000004000000}" name="lien"/>
     <tableColumn id="5" xr3:uid="{00000000-0010-0000-0000-000005000000}" name="sunoId"/>
+    <tableColumn id="6" xr3:uid="{00000000-0010-0000-0000-000006000000}" name="auteur"/>
   </tableColumns>
   <tableStyleInfo name="TableStyleMedium2" showFirstColumn="0" showLastColumn="0" showRowStripes="1" showColumnStripes="0"/>
 </table>
@@ -458,7 +468,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
-  <dimension ref="A1:E13"/>
+  <dimension ref="A1:F13"/>
   <sheetFormatPr baseColWidth="10" defaultColWidth="9.140625" defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="1" max="1" width="30" customWidth="1"/>
@@ -466,9 +476,10 @@
     <col min="3" max="3" width="13" customWidth="1"/>
     <col min="4" max="4" width="62" customWidth="1"/>
     <col min="5" max="5" width="40" customWidth="1"/>
+    <col min="6" max="6" width="20" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="1" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A1" t="s">
         <v>0</v>
       </c>
@@ -484,8 +495,11 @@
       <c r="E1" t="s">
         <v>4</v>
       </c>
-    </row>
-    <row r="2" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="F1" t="s">
+        <v>22</v>
+      </c>
+    </row>
+    <row r="2" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A2" t="s">
         <v>5</v>
       </c>
@@ -502,7 +516,7 @@
         <v>8</v>
       </c>
     </row>
-    <row r="3" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="3" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A3" t="s">
         <v>17</v>
       </c>
@@ -518,8 +532,11 @@
       <c r="E3" t="s">
         <v>16</v>
       </c>
-    </row>
-    <row r="4" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="F3" t="s">
+        <v>23</v>
+      </c>
+    </row>
+    <row r="4" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A4" t="s">
         <v>20</v>
       </c>
@@ -536,31 +553,31 @@
         <v>19</v>
       </c>
     </row>
-    <row r="5" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="5" spans="1:6" x14ac:dyDescent="0.25">
       <c r="C5" s="1"/>
     </row>
-    <row r="6" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="6" spans="1:6" x14ac:dyDescent="0.25">
       <c r="C6" s="1"/>
     </row>
-    <row r="7" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="7" spans="1:6" x14ac:dyDescent="0.25">
       <c r="C7" s="1"/>
     </row>
-    <row r="8" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="8" spans="1:6" x14ac:dyDescent="0.25">
       <c r="C8" s="1"/>
     </row>
-    <row r="9" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="9" spans="1:6" x14ac:dyDescent="0.25">
       <c r="C9" s="1"/>
     </row>
-    <row r="10" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="10" spans="1:6" x14ac:dyDescent="0.25">
       <c r="C10" s="1"/>
     </row>
-    <row r="11" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="11" spans="1:6" x14ac:dyDescent="0.25">
       <c r="C11" s="1"/>
     </row>
-    <row r="12" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="12" spans="1:6" x14ac:dyDescent="0.25">
       <c r="C12" s="1"/>
     </row>
-    <row r="13" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="13" spans="1:6" x14ac:dyDescent="0.25">
       <c r="C13" s="1"/>
     </row>
   </sheetData>
@@ -577,7 +594,7 @@
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0100-000000000000}">
-  <dimension ref="A1:A5"/>
+  <dimension ref="A1:A6"/>
   <sheetFormatPr baseColWidth="10" defaultColWidth="9.140625" defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="1" max="1" width="110" customWidth="1"/>
@@ -600,11 +617,16 @@
     </row>
     <row r="4" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A4" t="s">
-        <v>13</v>
+        <v>24</v>
       </c>
     </row>
     <row r="5" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A5" t="s">
+        <v>13</v>
+      </c>
+    </row>
+    <row r="6" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A6" t="s">
         <v>14</v>
       </c>
     </row>

</xml_diff>